<commit_message>
Use real product photos across the site
- Add 6 clean product photos to images/ (one per model), chosen to avoid
  supplier watermarks, alibaba URLs, and promo stickers in the source set
- Set the Image File column in product-data.xlsx (repo + OneDrive master)
- Show photos on detail-page hero and related cards (were SVG icons)
- Point publish.sh / memory at the relocated master: OneDrive/Stride-Website/

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product-data.xlsx
+++ b/product-data.xlsx
@@ -992,7 +992,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>q5.png</t>
+          <t>eco-e1.jpg</t>
         </is>
       </c>
       <c r="H3" s="45" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="G4" s="38" t="inlineStr">
         <is>
-          <t>q5.png</t>
+          <t>urban-u2.jpg</t>
         </is>
       </c>
       <c r="H4" s="43" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>q5.png</t>
+          <t>cruise-c3.jpg</t>
         </is>
       </c>
       <c r="H5" s="42" t="inlineStr">
@@ -1459,7 +1459,11 @@
       <c r="F6" s="39" t="n">
         <v>179000</v>
       </c>
-      <c r="G6" s="38" t="n"/>
+      <c r="G6" s="38" t="inlineStr">
+        <is>
+          <t>recline-r4.jpg</t>
+        </is>
+      </c>
       <c r="H6" s="43" t="inlineStr">
         <is>
           <t>Comfort meets reliability in the Recline R4. Designed for those who need more than just mobility, it features a manual reclining backrest for easy position adjustment, an adjustable footrest for added leg support, and an extended headrest that keeps you comfortably supported throughout the day. Simple, dependable, and built with everyday comfort in mind — the Recline R4 lets you move through your day and rest easy whenever you need to.</t>
@@ -1612,7 +1616,7 @@
       </c>
       <c r="G7" s="38" t="inlineStr">
         <is>
-          <t>q5.png</t>
+          <t>pr-x.jpg</t>
         </is>
       </c>
       <c r="H7" s="42" t="inlineStr">
@@ -1775,7 +1779,7 @@
       </c>
       <c r="G8" s="30" t="inlineStr">
         <is>
-          <t>q5.png</t>
+          <t>compact-air.jpg</t>
         </is>
       </c>
       <c r="H8" s="43" t="inlineStr">

</xml_diff>

<commit_message>
Add curated reviews and product photo galleries
Reviews: new optional `Reviews` sheet in product-data.xlsx (one row per
review) drives a "What customers say" section on each product page — gold
star summary, review cards, and AggregateRating/Review JSON-LD for rich
results. Generator degrades gracefully when the sheet is absent.

Galleries: switch the catalog to real studio photos and add a detail-page
image gallery. Each product shows a 3/4-front hero plus a thumbnail strip
(extra angles from the new optional `Gallery` sheet) that swaps the hero;
the product's `Image File` stays the card/compare image. Photos optimized
to ~1200px square JPGs; old single images removed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product-data.xlsx
+++ b/product-data.xlsx
@@ -7,6 +7,8 @@
     <sheet name="Guide" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Site Settings" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Lists" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Reviews" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gallery" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Products'!$A$2:$AI$10</definedName>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -92,8 +94,12 @@
       <color rgb="FF6B6E63"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -160,6 +166,11 @@
         <bgColor rgb="FFECEEE8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DE7356"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="7">
     <border/>
@@ -224,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -364,6 +375,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -992,7 +1006,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>eco-e1.jpg</t>
+          <t>eco-e1-1.jpg</t>
         </is>
       </c>
       <c r="H3" s="45" t="inlineStr">
@@ -1147,7 +1161,7 @@
       </c>
       <c r="G4" s="38" t="inlineStr">
         <is>
-          <t>urban-u2.jpg</t>
+          <t>urban-u2-1.jpg</t>
         </is>
       </c>
       <c r="H4" s="43" t="inlineStr">
@@ -1302,7 +1316,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>cruise-c3.jpg</t>
+          <t>cruise-c3-1.jpg</t>
         </is>
       </c>
       <c r="H5" s="42" t="inlineStr">
@@ -1461,7 +1475,7 @@
       </c>
       <c r="G6" s="38" t="inlineStr">
         <is>
-          <t>recline-r4.jpg</t>
+          <t>recline-r4-1.jpg</t>
         </is>
       </c>
       <c r="H6" s="43" t="inlineStr">
@@ -1616,7 +1630,7 @@
       </c>
       <c r="G7" s="38" t="inlineStr">
         <is>
-          <t>pr-x.jpg</t>
+          <t>pr-x-1.jpg</t>
         </is>
       </c>
       <c r="H7" s="42" t="inlineStr">
@@ -1779,7 +1793,7 @@
       </c>
       <c r="G8" s="30" t="inlineStr">
         <is>
-          <t>q5.png</t>
+          <t>compact-air-1.jpg</t>
         </is>
       </c>
       <c r="H8" s="43" t="inlineStr">
@@ -6759,4 +6773,412 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="46" min="1" max="1"/>
+    <col width="20" customWidth="1" style="46" min="2" max="2"/>
+    <col width="12" customWidth="1" style="46" min="3" max="3"/>
+    <col width="16" customWidth="1" style="46" min="4" max="4"/>
+    <col width="10" customWidth="1" style="46" min="5" max="5"/>
+    <col width="70" customWidth="1" style="46" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="54" t="inlineStr">
+        <is>
+          <t>Slug (URL id)</t>
+        </is>
+      </c>
+      <c r="B1" s="54" t="inlineStr">
+        <is>
+          <t>Customer Name</t>
+        </is>
+      </c>
+      <c r="C1" s="54" t="inlineStr">
+        <is>
+          <t>Rating (1-5)</t>
+        </is>
+      </c>
+      <c r="D1" s="54" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="E1" s="54" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F1" s="54" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>eco-e1</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>Imran Qureshi</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>Lahore</t>
+        </is>
+      </c>
+      <c r="E2" s="0" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="F2" s="0" t="inlineStr">
+        <is>
+          <t>Light enough to fold into my car boot on my own. Great value for the price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>eco-e1</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Sadia Khan</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>Islamabad</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>Reliable for daily indoor use and the delivery was quick. Battery lasts the full day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>urban-u2</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>Bilal Ahmed</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>Karachi</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>Handles broken footpaths around my area really well. The team answered every question on WhatsApp before I bought.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>recline-r4</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>Nadia Farooq</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>Rawalpindi</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>The recline makes a huge difference for my father's comfort on long sits. Build quality feels solid.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="46" min="1" max="1"/>
+    <col width="22" customWidth="1" style="46" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="54" t="inlineStr">
+        <is>
+          <t>Slug (URL id)</t>
+        </is>
+      </c>
+      <c r="B1" s="54" t="inlineStr">
+        <is>
+          <t>Image File</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>eco-e1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>eco-e1-2.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>eco-e1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>eco-e1-3.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>eco-e1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>eco-e1-4.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>urban-u2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>urban-u2-2.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>urban-u2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>urban-u2-3.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>urban-u2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>urban-u2-4.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>cruise-c3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>cruise-c3-2.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>cruise-c3</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>cruise-c3-3.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>cruise-c3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>cruise-c3-4.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>recline-r4</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>recline-r4-2.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>recline-r4</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>recline-r4-3.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>recline-r4</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>recline-r4-4.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>pr-x</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>pr-x-2.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>pr-x</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>pr-x-3.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>pr-x</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>pr-x-4.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>compact-air</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>compact-air-2.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>compact-air</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>compact-air-3.jpg</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Polish product UI and add a full SEO pass
UI/content:
- Product photos fill their (now square) containers; drop the padding/float.
- Add prev/next arrows to the detail-page gallery (wrap-around, arrow keys,
  synced with thumbnails).
- Move the category pill onto the card image (bottom-right overlay).
- Compare table highlights best values in green only (star removed; blurb
  updated to match).
- Remove em dashes (" —") from all visible copy.
- Update contact email to info@stridepakistan.com.
- Add site favicon (brand mark) across all pages.

SEO:
- Open Graph + Twitter Card + canonical tags on every page (rich link
  previews for WhatsApp/social).
- Clearer <title> tags on product pages.
- robots.txt and an auto-generated sitemap.xml.
- Structured data: Store (home), Product with price/availability +
  BreadcrumbList (product pages), plus existing reviews.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product-data.xlsx
+++ b/product-data.xlsx
@@ -1011,7 +1011,7 @@
       </c>
       <c r="H3" s="45" t="inlineStr">
         <is>
-          <t>An economical,  folding power chair with all the essential functionality — simple, reliable, and easy to carry in a car boot. Built for indoor use, and capable of working outdoors as well.</t>
+          <t>An economical,  folding power chair with all the essential functionality simple, reliable, and easy to carry in a car boot. Built for indoor use, and capable of working outdoors as well.</t>
         </is>
       </c>
       <c r="I3" s="34" t="inlineStr">
@@ -1081,12 +1081,12 @@
       </c>
       <c r="Z3" s="42" t="inlineStr">
         <is>
-          <t>An economical folding power chair with the everyday essentials — simple, reliable and easy to fold into a car boot. Built for indoor and light outdoor use.</t>
+          <t>An economical folding power chair with the everyday essentials simple, reliable and easy to fold into a car boot. Built for indoor and light outdoor use.</t>
         </is>
       </c>
       <c r="AA3" s="42" t="inlineStr">
         <is>
-          <t>An economical folding power chair with all the essentials — simple, reliable and easy to carry in a car boot. Built mainly for indoor use, it handles the outdoors too.</t>
+          <t>An economical folding power chair with all the essentials simple, reliable and easy to carry in a car boot. Built mainly for indoor use, it handles the outdoors too.</t>
         </is>
       </c>
       <c r="AB3" s="42" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="H4" s="43" t="inlineStr">
         <is>
-          <t>An affordable folding power chair that covers the everyday essentials — comfortable, dependable and easy to fold away. Great value for daily use at home and around town.</t>
+          <t>An affordable folding power chair that covers the everyday essentials comfortable, dependable and easy to fold away. Great value for daily use at home and around town.</t>
         </is>
       </c>
       <c r="I4" s="41" t="inlineStr">
@@ -1236,12 +1236,12 @@
       </c>
       <c r="Z4" s="43" t="inlineStr">
         <is>
-          <t>An affordable folding power chair with the everyday essentials — comfortable, dependable and easy to fold away. Great value for daily indoor and outdoor use.</t>
+          <t>An affordable folding power chair with the everyday essentials comfortable, dependable and easy to fold away. Great value for daily indoor and outdoor use.</t>
         </is>
       </c>
       <c r="AA4" s="43" t="inlineStr">
         <is>
-          <t>An affordable folding power chair that covers the everyday essentials — comfortable seating, responsive controls and a dependable battery, in a frame that folds away for easy storage and transport.</t>
+          <t>An affordable folding power chair that covers the everyday essentials comfortable seating, responsive controls and a dependable battery, in a frame that folds away for easy storage and transport.</t>
         </is>
       </c>
       <c r="AB4" s="43" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="H5" s="42" t="inlineStr">
         <is>
-          <t>Built to handle rough terrain without compromising on comfort. The Cruise C3 features rear wheel shocks that smooth out bumps and uneven ground, giving it standout outdoor capability few chairs in its class can match. Comfortable seating, responsive controls, and a dependable battery round out the experience — making it just as easy to rely on for everyday city life as it is for the rugged paths beyond it.</t>
+          <t>Built to handle rough terrain without compromising on comfort. The Cruise C3 features rear wheel shocks that smooth out bumps and uneven ground, giving it standout outdoor capability few chairs in its class can match. Comfortable seating, responsive controls, and a dependable battery round out the experience making it just as easy to rely on for everyday city life as it is for the rugged paths beyond it.</t>
         </is>
       </c>
       <c r="I5" s="34" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="Z5" s="42" t="inlineStr">
         <is>
-          <t>Built to handle rough terrain without compromising on comfort — rear-wheel shocks smooth out bumps and uneven ground for standout outdoor capability.</t>
+          <t>Built to handle rough terrain without compromising on comfort rear-wheel shocks smooth out bumps and uneven ground for standout outdoor capability.</t>
         </is>
       </c>
       <c r="AA5" s="42" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="H6" s="43" t="inlineStr">
         <is>
-          <t>Comfort meets reliability in the Recline R4. Designed for those who need more than just mobility, it features a manual reclining backrest for easy position adjustment, an adjustable footrest for added leg support, and an extended headrest that keeps you comfortably supported throughout the day. Simple, dependable, and built with everyday comfort in mind — the Recline R4 lets you move through your day and rest easy whenever you need to.</t>
+          <t>Comfort meets reliability in the Recline R4. Designed for those who need more than just mobility, it features a manual reclining backrest for easy position adjustment, an adjustable footrest for added leg support, and an extended headrest that keeps you comfortably supported throughout the day. Simple, dependable, and built with everyday comfort in mind the Recline R4 lets you move through your day and rest easy whenever you need to.</t>
         </is>
       </c>
       <c r="I6" s="41" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="Z6" s="43" t="inlineStr">
         <is>
-          <t>Comfort meets reliability in the Recline R4. Designed for those who need more than just mobility, it features a manual reclining backrest for easy position adjustment, an adjustable footrest for added leg support, and an extended headrest that keeps you comfortably supported throughout the day. Simple, dependable, and built with everyday comfort in mind — the Recline R4 lets you move through your day and rest easy whenever you need to.</t>
+          <t>Comfort meets reliability in the Recline R4. Designed for those who need more than just mobility, it features a manual reclining backrest for easy position adjustment, an adjustable footrest for added leg support, and an extended headrest that keeps you comfortably supported throughout the day. Simple, dependable, and built with everyday comfort in mind the Recline R4 lets you move through your day and rest easy whenever you need to.</t>
         </is>
       </c>
       <c r="AA6" s="43" t="inlineStr">
         <is>
-          <t>Comfort meets reliability in the Recline R4. A manual reclining backrest, adjustable footrest and extended headrest keep you comfortably supported through the day — simple, dependable and built with everyday comfort in mind.</t>
+          <t>Comfort meets reliability in the Recline R4. A manual reclining backrest, adjustable footrest and extended headrest keep you comfortably supported through the day simple, dependable and built with everyday comfort in mind.</t>
         </is>
       </c>
       <c r="AB6" s="43" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="H7" s="42" t="inlineStr">
         <is>
-          <t>Effortless comfort, powered by you. The PR- X features a power-operated reclining backrest and footrest, letting you adjust your position smoothly at the touch of a button — no manual effort required. An extended headrest adds complete support from head to toe, making it ideal for those who want maximum comfort with minimum effort. Simple to operate, dependable to rely on, and designed to help you rest exactly the way you want, whenever you need to.</t>
+          <t>Effortless comfort, powered by you. The PR- X features a power-operated reclining backrest and footrest, letting you adjust your position smoothly at the touch of a button no manual effort required. An extended headrest adds complete support from head to toe, making it ideal for those who want maximum comfort with minimum effort. Simple to operate, dependable to rely on, and designed to help you rest exactly the way you want, whenever you need to.</t>
         </is>
       </c>
       <c r="I7" s="41" t="inlineStr">
@@ -1713,12 +1713,12 @@
       </c>
       <c r="Z7" s="42" t="inlineStr">
         <is>
-          <t>Effortless comfort, powered by you. The PR-X features a power-operated reclining backrest and footrest, adjustable at the touch of a button — no manual effort required.</t>
+          <t>Effortless comfort, powered by you. The PR-X features a power-operated reclining backrest and footrest, adjustable at the touch of a button no manual effort required.</t>
         </is>
       </c>
       <c r="AA7" s="43" t="inlineStr">
         <is>
-          <t>Effortless comfort, powered by you. The PR-X's power-operated reclining backrest and footrest adjust at the touch of a button, and an extended headrest adds full support from head to toe — maximum comfort with minimum effort.</t>
+          <t>Effortless comfort, powered by you. The PR-X's power-operated reclining backrest and footrest adjust at the touch of a button, and an extended headrest adds full support from head to toe maximum comfort with minimum effort.</t>
         </is>
       </c>
       <c r="AB7" s="43" t="inlineStr">
@@ -1877,12 +1877,12 @@
       </c>
       <c r="AA8" s="43" t="inlineStr">
         <is>
-          <t>Just 26 kg and airline-friendly. The Compact Air folds in seconds and lifts easily — ideal for travel, hotels and getting in and out of a car without a struggle.</t>
+          <t>Just 26 kg and airline-friendly. The Compact Air folds in seconds and lifts easily ideal for travel, hotels and getting in and out of a car without a struggle.</t>
         </is>
       </c>
       <c r="AB8" s="43" t="inlineStr">
         <is>
-          <t>Only 26 kg — easy to lift</t>
+          <t>Only 26 kg easy to lift</t>
         </is>
       </c>
       <c r="AC8" s="43" t="inlineStr">
@@ -6975,204 +6975,204 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>eco-e1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>eco-e1-2.jpg</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>eco-e1</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>eco-e1-3.jpg</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>eco-e1</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>eco-e1-4.jpg</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>urban-u2</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>urban-u2-2.jpg</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>urban-u2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>urban-u2-3.jpg</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>urban-u2</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>urban-u2-4.jpg</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>cruise-c3</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>cruise-c3-2.jpg</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>cruise-c3</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>cruise-c3-3.jpg</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>cruise-c3</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>cruise-c3-4.jpg</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>recline-r4</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>recline-r4-2.jpg</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>recline-r4</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>recline-r4-3.jpg</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>recline-r4</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>recline-r4-4.jpg</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>pr-x</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>pr-x-2.jpg</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>pr-x</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>pr-x-3.jpg</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>pr-x</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>pr-x-4.jpg</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>compact-air</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>compact-air-2.jpg</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>compact-air</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>compact-air-3.jpg</t>
         </is>

</xml_diff>

<commit_message>
Update contact phone to +92 319 9464347 and hours
New number applied across Site Settings, generator defaults, index.html
(display, tel: and WhatsApp links, Store schema) and all regenerated
product pages and compare links. Business hours changed to
"Daily except Friday, 10am–7pm".

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product-data.xlsx
+++ b/product-data.xlsx
@@ -4587,6 +4587,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -4607,7 +4608,7 @@
       </c>
       <c r="B5" s="21" t="inlineStr">
         <is>
-          <t>+92 300 1234567</t>
+          <t>+92 319 9464347</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4620,7 @@
       </c>
       <c r="B6" s="21" t="inlineStr">
         <is>
-          <t>+92 300 1234567</t>
+          <t>+92 319 9464347</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4632,7 @@
       </c>
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>923001234567</t>
+          <t>923199464347</t>
         </is>
       </c>
     </row>
@@ -4643,7 +4644,7 @@
       </c>
       <c r="B8" s="21" t="inlineStr">
         <is>
-          <t>Sat–Thu, 10am–7pm</t>
+          <t>Daily except Friday, 10am–7pm</t>
         </is>
       </c>
     </row>

</xml_diff>